<commit_message>
Sending of RS485 subtype and CAN base ID added (not tested!)
</commit_message>
<xml_diff>
--- a/doc/VPT_SW_Requirements.xlsx
+++ b/doc/VPT_SW_Requirements.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\1_GitHub\vpt_npm\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\1_GitHub\vpt_npm\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A324E89-97B7-4AAB-882E-724ACDFB15E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9601472-CCED-4BD6-8713-27B6B1D094C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{B686515A-1D7B-4367-B1A5-D8A05F452FDA}"/>
   </bookViews>
@@ -456,9 +456,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -472,6 +469,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -481,60 +482,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF5FCD4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -576,82 +531,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF5FCD4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -998,681 +878,681 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="11"/>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="12"/>
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="C5" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="11"/>
-      <c r="B6" s="6" t="s">
+      <c r="A6" s="12"/>
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="11"/>
-      <c r="B7" s="6" t="s">
+      <c r="A7" s="12"/>
+      <c r="B7" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
-      <c r="B8" s="6" t="s">
+      <c r="A8" s="13"/>
+      <c r="B8" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+      <c r="A11" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="C14" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="12"/>
+      <c r="B16" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="12"/>
+      <c r="B17" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="12"/>
+      <c r="B18" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="12"/>
+      <c r="B19" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="13"/>
+      <c r="B20" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="11"/>
-      <c r="B16" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="11"/>
-      <c r="B17" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
-      <c r="B18" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="11"/>
-      <c r="B19" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="C19" s="14" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="12"/>
+      <c r="B22" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="12"/>
+      <c r="B23" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="12"/>
+      <c r="B24" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="12"/>
+      <c r="B25" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="12"/>
+      <c r="B26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="12"/>
+      <c r="B27" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="12"/>
+      <c r="B28" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="12"/>
+      <c r="B29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="13"/>
+      <c r="B30" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="12"/>
+      <c r="B32" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="13"/>
+      <c r="B33" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="12"/>
+      <c r="B37" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="12"/>
+      <c r="B38" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="12"/>
+      <c r="B39" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="12"/>
+      <c r="B40" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="12"/>
+      <c r="B41" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="12"/>
+      <c r="B42" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C42" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="12"/>
+      <c r="B43" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="12"/>
+      <c r="B44" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="12"/>
+      <c r="B45" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="12"/>
+      <c r="B46" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C46" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="12"/>
+      <c r="B47" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C47" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="12"/>
-      <c r="B20" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="14" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="12"/>
+      <c r="B48" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C48" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A49" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="C49" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="12"/>
+      <c r="B50" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="12"/>
+      <c r="B51" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C51" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="12"/>
+      <c r="B52" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="12"/>
+      <c r="B53" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="12"/>
+      <c r="B54" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="12"/>
+      <c r="B55" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="13"/>
+      <c r="B56" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C57" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="11"/>
-      <c r="B22" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="14" t="s">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="12"/>
+      <c r="B58" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="12"/>
+      <c r="B59" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="13"/>
+      <c r="B60" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C60" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="11"/>
-      <c r="B23" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="14" t="s">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B61" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C61" s="10" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="11"/>
-      <c r="B24" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="11"/>
-      <c r="B25" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="11"/>
-      <c r="B26" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="11"/>
-      <c r="B27" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="11"/>
-      <c r="B28" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="11"/>
-      <c r="B29" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C29" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="12"/>
-      <c r="B30" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="11"/>
-      <c r="B32" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C32" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="12"/>
-      <c r="B33" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C35" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="11"/>
-      <c r="B37" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C37" s="14" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="11"/>
-      <c r="B38" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C38" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="11"/>
-      <c r="B39" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="11"/>
-      <c r="B40" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="11"/>
-      <c r="B41" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="11"/>
-      <c r="B42" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="11"/>
-      <c r="B43" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="11"/>
-      <c r="B44" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="C44" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="11"/>
-      <c r="B45" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C45" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="11"/>
-      <c r="B46" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C46" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="11"/>
-      <c r="B47" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C47" s="14" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="12"/>
+      <c r="B62" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="13"/>
+      <c r="B63" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A64" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C65" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="11"/>
-      <c r="B48" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C48" s="14" t="s">
+    <row r="66" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A66" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C66" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A49" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B49" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="11"/>
-      <c r="B50" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="C50" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="11"/>
-      <c r="B51" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="11"/>
-      <c r="B52" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C52" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="11"/>
-      <c r="B53" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C53" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="11"/>
-      <c r="B54" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="11"/>
-      <c r="B55" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C55" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="12"/>
-      <c r="B56" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C56" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C57" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="11"/>
-      <c r="B58" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C58" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="11"/>
-      <c r="B59" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C59" s="14" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="12"/>
-      <c r="B60" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="C60" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C61" s="14" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="11"/>
-      <c r="B62" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="C62" s="14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="12"/>
-      <c r="B63" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A64" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B64" s="7" t="s">
-        <v>91</v>
-      </c>
-      <c r="C64" s="14" t="s">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="12"/>
+      <c r="B67" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C67" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B65" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C65" s="14" t="s">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="12"/>
+      <c r="B68" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A66" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B66" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C66" s="14" t="s">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="12"/>
+      <c r="B69" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C69" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="11"/>
-      <c r="B67" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C67" s="14" t="s">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="12"/>
+      <c r="B70" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C70" s="10" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="11"/>
-      <c r="B68" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C68" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="11"/>
-      <c r="B69" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C69" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="11"/>
-      <c r="B70" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="C70" s="14" t="s">
-        <v>95</v>
-      </c>
-    </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="12"/>
-      <c r="B71" s="6" t="s">
+      <c r="A71" s="13"/>
+      <c r="B71" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C71" s="14" t="s">
+      <c r="C71" s="10" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1690,24 +1570,24 @@
     <mergeCell ref="A36:A48"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C71">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="ToDo">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Postponed">
+      <formula>NOT(ISERROR(SEARCH("Postponed",C3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Rejected">
+      <formula>NOT(ISERROR(SEARCH("Rejected",C3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="ToDo">
       <formula>NOT(ISERROR(SEARCH("ToDo",C3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="ToDo">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="ToDo">
       <formula>NOT(ISERROR(SEARCH("ToDo",C3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="Done">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="Done">
       <formula>NOT(ISERROR(SEARCH("Done",C3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="Rejected">
-      <formula>NOT(ISERROR(SEARCH("Rejected",C3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Postponed">
-      <formula>NOT(ISERROR(SEARCH("Postponed",C3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C64:C71">
-    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="Rejected">
+    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="Rejected">
       <formula>NOT(ISERROR(SEARCH("Rejected",C64)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1726,27 +1606,27 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>96</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SW requirements table updated
</commit_message>
<xml_diff>
--- a/doc/VPT_SW_Requirements.xlsx
+++ b/doc/VPT_SW_Requirements.xlsx
@@ -432,52 +432,56 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -609,685 +613,685 @@
   <sheetFormatPr defaultColWidth="10.79296875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="78.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="78.45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" s="6" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" s="7" customFormat="true" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="7" t="s">
+      <c r="A5" s="4"/>
+      <c r="B5" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3"/>
-      <c r="B6" s="7" t="s">
+      <c r="A6" s="4"/>
+      <c r="B6" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3"/>
-      <c r="B7" s="7" t="s">
+      <c r="A7" s="4"/>
+      <c r="B7" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3"/>
-      <c r="B8" s="7" t="s">
+      <c r="A8" s="4"/>
+      <c r="B8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="B14" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="4"/>
+      <c r="B17" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="4"/>
+      <c r="B18" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3"/>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="4"/>
+      <c r="B19" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3"/>
-      <c r="B20" s="9" t="s">
+      <c r="A20" s="4"/>
+      <c r="B20" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+      <c r="A21" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>9</v>
+      <c r="C21" s="6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="7" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-      <c r="B23" s="7" t="s">
+      <c r="A23" s="4"/>
+      <c r="B23" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3"/>
-      <c r="B24" s="7" t="s">
+      <c r="A24" s="4"/>
+      <c r="B24" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3"/>
-      <c r="B25" s="7" t="s">
+      <c r="A25" s="4"/>
+      <c r="B25" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3"/>
-      <c r="B26" s="7" t="s">
+      <c r="A26" s="4"/>
+      <c r="B26" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3"/>
-      <c r="B27" s="7" t="s">
+      <c r="A27" s="4"/>
+      <c r="B27" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3"/>
-      <c r="B28" s="7" t="s">
+      <c r="A28" s="4"/>
+      <c r="B28" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3"/>
-      <c r="B29" s="7" t="s">
+      <c r="A29" s="4"/>
+      <c r="B29" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-      <c r="B30" s="7" t="s">
+      <c r="A30" s="4"/>
+      <c r="B30" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="A31" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B31" s="7" t="s">
+      <c r="B31" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>9</v>
+      <c r="C31" s="6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3"/>
-      <c r="B32" s="7" t="s">
+      <c r="A32" s="4"/>
+      <c r="B32" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>9</v>
+      <c r="C32" s="6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
-      <c r="B33" s="7" t="s">
+      <c r="A33" s="4"/>
+      <c r="B33" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>9</v>
+      <c r="C33" s="6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="A34" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
+      <c r="A35" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B36" s="8" t="s">
+      <c r="B36" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="10"/>
-      <c r="B37" s="7" t="s">
+      <c r="A37" s="11"/>
+      <c r="B37" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="10"/>
-      <c r="B38" s="7" t="s">
+      <c r="A38" s="11"/>
+      <c r="B38" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="10"/>
-      <c r="B39" s="7" t="s">
+      <c r="A39" s="11"/>
+      <c r="B39" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="10"/>
-      <c r="B40" s="7" t="s">
+      <c r="A40" s="11"/>
+      <c r="B40" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="10"/>
-      <c r="B41" s="7" t="s">
+      <c r="A41" s="11"/>
+      <c r="B41" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="10"/>
-      <c r="B42" s="7" t="s">
+      <c r="A42" s="11"/>
+      <c r="B42" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10"/>
-      <c r="B43" s="7" t="s">
+      <c r="A43" s="11"/>
+      <c r="B43" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="10"/>
-      <c r="B44" s="7" t="s">
+      <c r="A44" s="11"/>
+      <c r="B44" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="10"/>
-      <c r="B45" s="7" t="s">
+      <c r="A45" s="11"/>
+      <c r="B45" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="10"/>
-      <c r="B46" s="7" t="s">
+      <c r="A46" s="11"/>
+      <c r="B46" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10"/>
-      <c r="B47" s="7" t="s">
+      <c r="A47" s="11"/>
+      <c r="B47" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="10"/>
-      <c r="B48" s="7" t="s">
+      <c r="A48" s="11"/>
+      <c r="B48" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="3" t="s">
+      <c r="A49" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C49" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3"/>
-      <c r="B50" s="7" t="s">
+      <c r="A50" s="4"/>
+      <c r="B50" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3"/>
-      <c r="B51" s="7" t="s">
+      <c r="A51" s="4"/>
+      <c r="B51" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="3"/>
-      <c r="B52" s="7" t="s">
+      <c r="A52" s="4"/>
+      <c r="B52" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3"/>
-      <c r="B53" s="7" t="s">
+      <c r="A53" s="4"/>
+      <c r="B53" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3"/>
-      <c r="B54" s="7" t="s">
+      <c r="A54" s="4"/>
+      <c r="B54" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3"/>
-      <c r="B55" s="7" t="s">
+      <c r="A55" s="4"/>
+      <c r="B55" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3"/>
-      <c r="B56" s="7" t="s">
+      <c r="A56" s="4"/>
+      <c r="B56" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C56" s="5" t="s">
+      <c r="C56" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="A57" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="C57" s="5" t="s">
-        <v>9</v>
+      <c r="C57" s="6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3"/>
-      <c r="B58" s="7" t="s">
+      <c r="A58" s="4"/>
+      <c r="B58" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="C58" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3"/>
-      <c r="B59" s="7" t="s">
+      <c r="A59" s="4"/>
+      <c r="B59" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C59" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="3"/>
-      <c r="B60" s="7" t="s">
+      <c r="A60" s="4"/>
+      <c r="B60" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
+      <c r="A61" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="C61" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3"/>
-      <c r="B62" s="7" t="s">
+      <c r="A62" s="4"/>
+      <c r="B62" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="C62" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3"/>
-      <c r="B63" s="7" t="s">
+      <c r="A63" s="4"/>
+      <c r="B63" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="C63" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3" t="s">
+      <c r="A64" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B64" s="8" t="s">
+      <c r="B64" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="C64" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="3" t="s">
+      <c r="A65" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B65" s="7" t="s">
+      <c r="B65" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="C65" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="28.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="3" t="s">
+      <c r="A66" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B66" s="8" t="s">
+      <c r="B66" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="C66" s="5" t="s">
+      <c r="C66" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3"/>
-      <c r="B67" s="7" t="s">
+      <c r="A67" s="4"/>
+      <c r="B67" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="C67" s="5" t="s">
+      <c r="C67" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="3"/>
-      <c r="B68" s="7" t="s">
+      <c r="A68" s="4"/>
+      <c r="B68" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="C68" s="5" t="s">
+      <c r="C68" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3"/>
-      <c r="B69" s="7" t="s">
+      <c r="A69" s="4"/>
+      <c r="B69" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="C69" s="5" t="s">
+      <c r="C69" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3"/>
-      <c r="B70" s="7" t="s">
+      <c r="A70" s="4"/>
+      <c r="B70" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="C70" s="5" t="s">
+      <c r="C70" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3"/>
-      <c r="B71" s="7" t="s">
+      <c r="A71" s="4"/>
+      <c r="B71" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="C71" s="5" t="s">
+      <c r="C71" s="6" t="s">
         <v>34</v>
       </c>
     </row>
@@ -1351,27 +1355,27 @@
   <sheetFormatPr defaultColWidth="10.79296875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="8" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="8" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="8" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>